<commit_message>
Update PDP tender outputs
</commit_message>
<xml_diff>
--- a/outputs/pdp_tenders_latest.xlsx
+++ b/outputs/pdp_tenders_latest.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>['https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-01#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-02#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-03#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-04#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-05#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-06#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-07#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-08#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-09#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-10#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-11#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-12#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-13#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-14#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-15#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-16#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-17#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-18#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-19#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-20#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-21#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-22#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-23#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-24#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-25#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-26#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-27#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-28#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-29#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-30#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-31#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-32#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-33#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-34#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-35#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-36#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-37#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-38#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-39#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-40#publish-filter']</t>
+          <t>['https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-01#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-02#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-03#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-04#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-05#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-06#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-07#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-08#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-09#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-10#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-11#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-12#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-13#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-14#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-15#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-16#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-17#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-18#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-19#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-20#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-21#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-22#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-23#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-24#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-25#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-26#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-27#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-28#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-29#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-30#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-31#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-32#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-33#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-34#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-35#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-36#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-37#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-38#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-39#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-40#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-41#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-42#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-43#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-44#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-45#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-46#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-47#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-48#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-49#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-50#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-51#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-52#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-53#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-54#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-55#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-56#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-57#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-58#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-59#publish-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-60#publish-filter']</t>
         </is>
       </c>
       <c r="P39" t="n">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>['https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-01#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-02#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-03#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-04#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-05#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-06#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-07#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-08#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-09#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-10#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-11#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-12#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-13#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-14#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-15#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-16#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-17#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-18#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-19#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-20#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-21#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-22#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-23#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-24#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-25#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-26#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-27#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-28#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-29#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-30#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-31#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-32#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-33#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-34#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-35#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-36#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-37#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-38#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-39#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-40#cats-filter']</t>
+          <t>['https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-01#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-02#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-03#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-04#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-05#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-06#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-07#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-08#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-09#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-10#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-11#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-12#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-13#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-14#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-15#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-16#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-17#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-18#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-19#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-20#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-21#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-22#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-23#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-24#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-25#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-26#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-27#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-28#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-29#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-30#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-31#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-32#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-33#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-34#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-35#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-36#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-37#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-38#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-39#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-40#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-41#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-42#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-43#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-44#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-45#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-46#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-47#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-48#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-49#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-50#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-51#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-52#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-53#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-54#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-55#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-56#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-57#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-58#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-59#cats-filter', 'https://www.hezarehinfo.net/tenders/-!/pfrom-1405-04-17/pto-1405-04-18/page-60#cats-filter']</t>
         </is>
       </c>
       <c r="P40" t="n">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:46+00:00</t>
+          <t>2026-07-09T11:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -4787,7 +4787,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4866,7 @@
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5577,7 +5577,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -6209,7 +6209,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:49+00:00</t>
+          <t>2026-07-09T11:27:24+00:00</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6371,7 +6371,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6450,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -7082,7 +7082,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -7236,7 +7236,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:52+00:00</t>
+          <t>2026-07-09T11:27:27+00:00</t>
         </is>
       </c>
     </row>
@@ -7315,7 +7315,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7394,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7473,7 +7473,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7552,7 +7552,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7710,7 +7710,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7789,7 +7789,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7947,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8184,7 +8184,7 @@
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8263,7 @@
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8421,7 +8421,7 @@
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8579,7 @@
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8658,7 +8658,7 @@
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8816,7 +8816,7 @@
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:55+00:00</t>
+          <t>2026-07-09T11:27:30+00:00</t>
         </is>
       </c>
     </row>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8970,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9365,7 +9365,7 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9677,7 +9677,7 @@
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9756,7 +9756,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9831,7 +9831,7 @@
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9910,7 +9910,7 @@
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -9989,7 +9989,7 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10068,7 +10068,7 @@
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10222,7 @@
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10301,7 +10301,7 @@
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>2026-07-09T10:12:58+00:00</t>
+          <t>2026-07-09T11:27:33+00:00</t>
         </is>
       </c>
     </row>
@@ -10459,7 +10459,7 @@
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10538,7 @@
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10617,7 +10617,7 @@
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10775,7 @@
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10854,7 +10854,7 @@
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -10933,7 +10933,7 @@
       </c>
       <c r="S137" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11012,7 +11012,7 @@
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11091,7 +11091,7 @@
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11249,7 +11249,7 @@
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11328,7 +11328,7 @@
       </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11407,7 +11407,7 @@
       </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11486,7 +11486,7 @@
       </c>
       <c r="S144" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11565,7 +11565,7 @@
       </c>
       <c r="S145" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11644,7 +11644,7 @@
       </c>
       <c r="S146" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="S147" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11802,7 +11802,7 @@
       </c>
       <c r="S148" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11881,7 +11881,7 @@
       </c>
       <c r="S149" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -11960,7 +11960,7 @@
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:01+00:00</t>
+          <t>2026-07-09T11:27:38+00:00</t>
         </is>
       </c>
     </row>
@@ -12039,7 +12039,7 @@
       </c>
       <c r="S151" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12118,7 +12118,7 @@
       </c>
       <c r="S152" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12193,7 +12193,7 @@
       </c>
       <c r="S153" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12272,7 +12272,7 @@
       </c>
       <c r="S154" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12351,7 +12351,7 @@
       </c>
       <c r="S155" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12430,7 +12430,7 @@
       </c>
       <c r="S156" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12509,7 +12509,7 @@
       </c>
       <c r="S157" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12588,7 +12588,7 @@
       </c>
       <c r="S158" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12667,7 +12667,7 @@
       </c>
       <c r="S159" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12742,7 +12742,7 @@
       </c>
       <c r="S160" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12821,7 +12821,7 @@
       </c>
       <c r="S161" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="S162" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -12971,7 +12971,7 @@
       </c>
       <c r="S163" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13046,7 @@
       </c>
       <c r="S164" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13125,7 +13125,7 @@
       </c>
       <c r="S165" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="S166" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13283,7 +13283,7 @@
       </c>
       <c r="S167" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13362,7 +13362,7 @@
       </c>
       <c r="S168" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="S169" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13520,7 +13520,7 @@
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:03+00:00</t>
+          <t>2026-07-09T11:27:41+00:00</t>
         </is>
       </c>
     </row>
@@ -13599,7 +13599,7 @@
       </c>
       <c r="S171" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13674,7 +13674,7 @@
       </c>
       <c r="S172" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13753,7 +13753,7 @@
       </c>
       <c r="S173" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13828,7 +13828,7 @@
       </c>
       <c r="S174" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13907,7 +13907,7 @@
       </c>
       <c r="S175" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -13982,7 +13982,7 @@
       </c>
       <c r="S176" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14061,7 +14061,7 @@
       </c>
       <c r="S177" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14140,7 +14140,7 @@
       </c>
       <c r="S178" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14215,7 +14215,7 @@
       </c>
       <c r="S179" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="S180" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14365,7 +14365,7 @@
       </c>
       <c r="S181" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14444,7 +14444,7 @@
       </c>
       <c r="S182" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14523,7 +14523,7 @@
       </c>
       <c r="S183" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14598,7 +14598,7 @@
       </c>
       <c r="S184" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14673,7 +14673,7 @@
       </c>
       <c r="S185" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14752,7 +14752,7 @@
       </c>
       <c r="S186" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14831,7 +14831,7 @@
       </c>
       <c r="S187" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14910,7 +14910,7 @@
       </c>
       <c r="S188" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -14989,7 +14989,7 @@
       </c>
       <c r="S189" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:06+00:00</t>
+          <t>2026-07-09T11:27:45+00:00</t>
         </is>
       </c>
     </row>
@@ -15068,7 +15068,7 @@
       </c>
       <c r="S190" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15147,7 +15147,7 @@
       </c>
       <c r="S191" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15226,7 +15226,7 @@
       </c>
       <c r="S192" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="S193" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15384,7 +15384,7 @@
       </c>
       <c r="S194" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15463,7 +15463,7 @@
       </c>
       <c r="S195" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15542,7 +15542,7 @@
       </c>
       <c r="S196" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15621,7 +15621,7 @@
       </c>
       <c r="S197" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15700,7 +15700,7 @@
       </c>
       <c r="S198" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15779,7 +15779,7 @@
       </c>
       <c r="S199" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15858,7 +15858,7 @@
       </c>
       <c r="S200" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -15937,7 +15937,7 @@
       </c>
       <c r="S201" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16012,7 +16012,7 @@
       </c>
       <c r="S202" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="S203" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16170,7 +16170,7 @@
       </c>
       <c r="S204" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16245,7 +16245,7 @@
       </c>
       <c r="S205" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16324,7 +16324,7 @@
       </c>
       <c r="S206" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16403,7 +16403,7 @@
       </c>
       <c r="S207" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16482,7 +16482,7 @@
       </c>
       <c r="S208" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16561,7 +16561,7 @@
       </c>
       <c r="S209" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:09+00:00</t>
+          <t>2026-07-09T11:27:48+00:00</t>
         </is>
       </c>
     </row>
@@ -16640,7 +16640,7 @@
       </c>
       <c r="S210" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -16715,7 +16715,7 @@
       </c>
       <c r="S211" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -16794,7 +16794,7 @@
       </c>
       <c r="S212" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -16873,7 +16873,7 @@
       </c>
       <c r="S213" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -16952,7 +16952,7 @@
       </c>
       <c r="S214" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17031,7 +17031,7 @@
       </c>
       <c r="S215" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17110,7 +17110,7 @@
       </c>
       <c r="S216" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17189,7 +17189,7 @@
       </c>
       <c r="S217" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17264,7 +17264,7 @@
       </c>
       <c r="S218" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17343,7 +17343,7 @@
       </c>
       <c r="S219" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17418,7 +17418,7 @@
       </c>
       <c r="S220" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="S221" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17576,7 +17576,7 @@
       </c>
       <c r="S222" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17655,7 +17655,7 @@
       </c>
       <c r="S223" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17734,7 +17734,7 @@
       </c>
       <c r="S224" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17813,7 +17813,7 @@
       </c>
       <c r="S225" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17888,7 +17888,7 @@
       </c>
       <c r="S226" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -17967,7 +17967,7 @@
       </c>
       <c r="S227" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -18046,7 +18046,7 @@
       </c>
       <c r="S228" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:11+00:00</t>
+          <t>2026-07-09T11:27:52+00:00</t>
         </is>
       </c>
     </row>
@@ -18125,7 +18125,7 @@
       </c>
       <c r="S229" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18200,7 +18200,7 @@
       </c>
       <c r="S230" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18275,7 +18275,7 @@
       </c>
       <c r="S231" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18354,7 +18354,7 @@
       </c>
       <c r="S232" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18433,7 +18433,7 @@
       </c>
       <c r="S233" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18508,7 +18508,7 @@
       </c>
       <c r="S234" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18583,7 +18583,7 @@
       </c>
       <c r="S235" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18662,7 +18662,7 @@
       </c>
       <c r="S236" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18741,7 +18741,7 @@
       </c>
       <c r="S237" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18820,7 +18820,7 @@
       </c>
       <c r="S238" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18899,7 +18899,7 @@
       </c>
       <c r="S239" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -18978,7 +18978,7 @@
       </c>
       <c r="S240" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19057,7 +19057,7 @@
       </c>
       <c r="S241" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19136,7 +19136,7 @@
       </c>
       <c r="S242" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19215,7 +19215,7 @@
       </c>
       <c r="S243" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19294,7 +19294,7 @@
       </c>
       <c r="S244" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19373,7 +19373,7 @@
       </c>
       <c r="S245" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19452,7 +19452,7 @@
       </c>
       <c r="S246" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19531,7 +19531,7 @@
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19606,7 +19606,7 @@
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:13+00:00</t>
+          <t>2026-07-09T11:27:54+00:00</t>
         </is>
       </c>
     </row>
@@ -19685,7 +19685,7 @@
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -19843,7 +19843,7 @@
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -19922,7 +19922,7 @@
       </c>
       <c r="S252" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20001,7 +20001,7 @@
       </c>
       <c r="S253" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20080,7 +20080,7 @@
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20159,7 @@
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20238,7 +20238,7 @@
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20317,7 +20317,7 @@
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20396,7 +20396,7 @@
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20475,7 +20475,7 @@
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20554,7 +20554,7 @@
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20629,7 +20629,7 @@
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20708,7 +20708,7 @@
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20787,7 +20787,7 @@
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20862,7 +20862,7 @@
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -20941,7 +20941,7 @@
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -21016,7 +21016,7 @@
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -21091,7 +21091,7 @@
       </c>
       <c r="S267" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -21170,7 +21170,7 @@
       </c>
       <c r="S268" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:16+00:00</t>
+          <t>2026-07-09T11:27:57+00:00</t>
         </is>
       </c>
     </row>
@@ -21249,7 +21249,7 @@
       </c>
       <c r="S269" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21328,7 +21328,7 @@
       </c>
       <c r="S270" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="S271" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21486,7 +21486,7 @@
       </c>
       <c r="S272" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21565,7 +21565,7 @@
       </c>
       <c r="S273" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21640,7 +21640,7 @@
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21719,7 +21719,7 @@
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21794,7 +21794,7 @@
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21869,7 +21869,7 @@
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -21948,7 +21948,7 @@
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22027,7 +22027,7 @@
       </c>
       <c r="S279" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22106,7 +22106,7 @@
       </c>
       <c r="S280" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22181,7 +22181,7 @@
       </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22260,7 +22260,7 @@
       </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22339,7 +22339,7 @@
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22418,7 +22418,7 @@
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22497,7 +22497,7 @@
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22576,7 +22576,7 @@
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22655,7 +22655,7 @@
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22734,7 +22734,7 @@
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:19+00:00</t>
+          <t>2026-07-09T11:27:59+00:00</t>
         </is>
       </c>
     </row>
@@ -22813,7 +22813,7 @@
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -22892,7 +22892,7 @@
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -22971,7 +22971,7 @@
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23050,7 +23050,7 @@
       </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23129,7 +23129,7 @@
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23208,7 +23208,7 @@
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23287,7 +23287,7 @@
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23366,7 +23366,7 @@
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23445,7 +23445,7 @@
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23520,7 +23520,7 @@
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23599,7 +23599,7 @@
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23674,7 +23674,7 @@
       </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23753,7 +23753,7 @@
       </c>
       <c r="S301" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23832,7 +23832,7 @@
       </c>
       <c r="S302" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23911,7 +23911,7 @@
       </c>
       <c r="S303" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -23990,7 +23990,7 @@
       </c>
       <c r="S304" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -24069,7 +24069,7 @@
       </c>
       <c r="S305" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -24144,7 +24144,7 @@
       </c>
       <c r="S306" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -24223,7 +24223,7 @@
       </c>
       <c r="S307" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -24302,7 +24302,7 @@
       </c>
       <c r="S308" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:21+00:00</t>
+          <t>2026-07-09T11:28:02+00:00</t>
         </is>
       </c>
     </row>
@@ -24381,7 +24381,7 @@
       </c>
       <c r="S309" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24460,7 +24460,7 @@
       </c>
       <c r="S310" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24539,7 +24539,7 @@
       </c>
       <c r="S311" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24618,7 +24618,7 @@
       </c>
       <c r="S312" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24697,7 +24697,7 @@
       </c>
       <c r="S313" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24776,7 +24776,7 @@
       </c>
       <c r="S314" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24855,7 +24855,7 @@
       </c>
       <c r="S315" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -24934,7 +24934,7 @@
       </c>
       <c r="S316" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25013,7 +25013,7 @@
       </c>
       <c r="S317" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25092,7 +25092,7 @@
       </c>
       <c r="S318" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25171,7 +25171,7 @@
       </c>
       <c r="S319" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25250,7 +25250,7 @@
       </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25329,7 +25329,7 @@
       </c>
       <c r="S321" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25408,7 +25408,7 @@
       </c>
       <c r="S322" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25487,7 +25487,7 @@
       </c>
       <c r="S323" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25566,7 +25566,7 @@
       </c>
       <c r="S324" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25645,7 +25645,7 @@
       </c>
       <c r="S325" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25724,7 +25724,7 @@
       </c>
       <c r="S326" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25803,7 +25803,7 @@
       </c>
       <c r="S327" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25882,7 +25882,7 @@
       </c>
       <c r="S328" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:24+00:00</t>
+          <t>2026-07-09T11:28:06+00:00</t>
         </is>
       </c>
     </row>
@@ -25961,7 +25961,7 @@
       </c>
       <c r="S329" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26040,7 +26040,7 @@
       </c>
       <c r="S330" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26119,7 +26119,7 @@
       </c>
       <c r="S331" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26198,7 +26198,7 @@
       </c>
       <c r="S332" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26277,7 +26277,7 @@
       </c>
       <c r="S333" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26352,7 +26352,7 @@
       </c>
       <c r="S334" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26431,7 +26431,7 @@
       </c>
       <c r="S335" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26510,7 +26510,7 @@
       </c>
       <c r="S336" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26585,7 +26585,7 @@
       </c>
       <c r="S337" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26664,7 +26664,7 @@
       </c>
       <c r="S338" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26739,7 +26739,7 @@
       </c>
       <c r="S339" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26814,7 +26814,7 @@
       </c>
       <c r="S340" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26893,7 +26893,7 @@
       </c>
       <c r="S341" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -26968,7 +26968,7 @@
       </c>
       <c r="S342" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -27047,7 +27047,7 @@
       </c>
       <c r="S343" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -27122,7 +27122,7 @@
       </c>
       <c r="S344" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -27201,7 +27201,7 @@
       </c>
       <c r="S345" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:27+00:00</t>
+          <t>2026-07-09T11:28:10+00:00</t>
         </is>
       </c>
     </row>
@@ -27280,7 +27280,7 @@
       </c>
       <c r="S346" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27355,7 +27355,7 @@
       </c>
       <c r="S347" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27430,7 +27430,7 @@
       </c>
       <c r="S348" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27509,7 +27509,7 @@
       </c>
       <c r="S349" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27588,7 +27588,7 @@
       </c>
       <c r="S350" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27667,7 +27667,7 @@
       </c>
       <c r="S351" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27746,7 +27746,7 @@
       </c>
       <c r="S352" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27821,7 +27821,7 @@
       </c>
       <c r="S353" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27900,7 +27900,7 @@
       </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -27979,7 +27979,7 @@
       </c>
       <c r="S355" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28058,7 +28058,7 @@
       </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28133,7 +28133,7 @@
       </c>
       <c r="S357" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28212,7 +28212,7 @@
       </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28291,7 +28291,7 @@
       </c>
       <c r="S359" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28370,7 +28370,7 @@
       </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28449,7 +28449,7 @@
       </c>
       <c r="S361" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28524,7 +28524,7 @@
       </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28603,7 +28603,7 @@
       </c>
       <c r="S363" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28682,7 +28682,7 @@
       </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:30+00:00</t>
+          <t>2026-07-09T11:28:14+00:00</t>
         </is>
       </c>
     </row>
@@ -28761,7 +28761,7 @@
       </c>
       <c r="S365" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -28840,7 +28840,7 @@
       </c>
       <c r="S366" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -28919,7 +28919,7 @@
       </c>
       <c r="S367" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -28998,7 +28998,7 @@
       </c>
       <c r="S368" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29077,7 +29077,7 @@
       </c>
       <c r="S369" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29156,7 +29156,7 @@
       </c>
       <c r="S370" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29235,7 +29235,7 @@
       </c>
       <c r="S371" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29314,7 +29314,7 @@
       </c>
       <c r="S372" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29393,7 +29393,7 @@
       </c>
       <c r="S373" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29472,7 +29472,7 @@
       </c>
       <c r="S374" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29551,7 +29551,7 @@
       </c>
       <c r="S375" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29630,7 +29630,7 @@
       </c>
       <c r="S376" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29709,7 +29709,7 @@
       </c>
       <c r="S377" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29788,7 +29788,7 @@
       </c>
       <c r="S378" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29867,7 +29867,7 @@
       </c>
       <c r="S379" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -29946,7 +29946,7 @@
       </c>
       <c r="S380" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -30025,7 +30025,7 @@
       </c>
       <c r="S381" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -30104,7 +30104,7 @@
       </c>
       <c r="S382" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:33+00:00</t>
+          <t>2026-07-09T11:28:18+00:00</t>
         </is>
       </c>
     </row>
@@ -30183,7 +30183,7 @@
       </c>
       <c r="S383" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30262,7 +30262,7 @@
       </c>
       <c r="S384" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30341,7 +30341,7 @@
       </c>
       <c r="S385" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30420,7 +30420,7 @@
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30499,7 +30499,7 @@
       </c>
       <c r="S387" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30578,7 +30578,7 @@
       </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30657,7 +30657,7 @@
       </c>
       <c r="S389" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30736,7 +30736,7 @@
       </c>
       <c r="S390" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30815,7 +30815,7 @@
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30894,7 +30894,7 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -30969,7 +30969,7 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31044,7 +31044,7 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31123,7 +31123,7 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31202,7 +31202,7 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31281,7 +31281,7 @@
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31360,7 +31360,7 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31439,7 +31439,7 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31514,7 +31514,7 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31593,7 +31593,7 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:36+00:00</t>
+          <t>2026-07-09T11:28:22+00:00</t>
         </is>
       </c>
     </row>
@@ -31672,7 +31672,7 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -31751,7 +31751,7 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -31826,7 +31826,7 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -31905,7 +31905,7 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -31980,7 +31980,7 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32059,7 +32059,7 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32138,7 +32138,7 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32217,7 +32217,7 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32296,7 +32296,7 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32375,7 +32375,7 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32454,7 +32454,7 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32533,7 +32533,7 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32608,7 +32608,7 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32687,7 +32687,7 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32766,7 +32766,7 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32845,7 +32845,7 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -32924,7 +32924,7 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -33003,7 +33003,7 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -33082,7 +33082,7 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -33161,7 +33161,7 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:39+00:00</t>
+          <t>2026-07-09T11:28:25+00:00</t>
         </is>
       </c>
     </row>
@@ -33240,7 +33240,7 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33319,7 +33319,7 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33398,7 +33398,7 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33477,7 +33477,7 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33556,7 +33556,7 @@
       </c>
       <c r="S426" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33635,7 +33635,7 @@
       </c>
       <c r="S427" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33714,7 +33714,7 @@
       </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33793,7 +33793,7 @@
       </c>
       <c r="S429" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33872,7 +33872,7 @@
       </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -33951,7 +33951,7 @@
       </c>
       <c r="S431" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34030,7 +34030,7 @@
       </c>
       <c r="S432" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34109,7 +34109,7 @@
       </c>
       <c r="S433" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34188,7 +34188,7 @@
       </c>
       <c r="S434" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34267,7 +34267,7 @@
       </c>
       <c r="S435" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34346,7 +34346,7 @@
       </c>
       <c r="S436" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34425,7 +34425,7 @@
       </c>
       <c r="S437" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34500,7 +34500,7 @@
       </c>
       <c r="S438" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34575,7 +34575,7 @@
       </c>
       <c r="S439" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:42+00:00</t>
+          <t>2026-07-09T11:28:28+00:00</t>
         </is>
       </c>
     </row>
@@ -34654,7 +34654,7 @@
       </c>
       <c r="S440" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -34729,7 +34729,7 @@
       </c>
       <c r="S441" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -34804,7 +34804,7 @@
       </c>
       <c r="S442" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -34879,7 +34879,7 @@
       </c>
       <c r="S443" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -34958,7 +34958,7 @@
       </c>
       <c r="S444" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35037,7 +35037,7 @@
       </c>
       <c r="S445" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35116,7 +35116,7 @@
       </c>
       <c r="S446" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35195,7 +35195,7 @@
       </c>
       <c r="S447" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35274,7 +35274,7 @@
       </c>
       <c r="S448" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35349,7 +35349,7 @@
       </c>
       <c r="S449" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35428,7 +35428,7 @@
       </c>
       <c r="S450" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35503,7 +35503,7 @@
       </c>
       <c r="S451" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35578,7 +35578,7 @@
       </c>
       <c r="S452" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35657,7 +35657,7 @@
       </c>
       <c r="S453" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35736,7 +35736,7 @@
       </c>
       <c r="S454" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35811,7 +35811,7 @@
       </c>
       <c r="S455" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35890,7 +35890,7 @@
       </c>
       <c r="S456" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -35965,7 +35965,7 @@
       </c>
       <c r="S457" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -36044,7 +36044,7 @@
       </c>
       <c r="S458" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:45+00:00</t>
+          <t>2026-07-09T11:28:32+00:00</t>
         </is>
       </c>
     </row>
@@ -36123,7 +36123,7 @@
       </c>
       <c r="S459" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36202,7 +36202,7 @@
       </c>
       <c r="S460" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36281,7 +36281,7 @@
       </c>
       <c r="S461" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36360,7 +36360,7 @@
       </c>
       <c r="S462" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36439,7 +36439,7 @@
       </c>
       <c r="S463" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36518,7 +36518,7 @@
       </c>
       <c r="S464" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36593,7 +36593,7 @@
       </c>
       <c r="S465" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36672,7 +36672,7 @@
       </c>
       <c r="S466" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36751,7 +36751,7 @@
       </c>
       <c r="S467" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36830,7 +36830,7 @@
       </c>
       <c r="S468" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36909,7 +36909,7 @@
       </c>
       <c r="S469" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -36988,7 +36988,7 @@
       </c>
       <c r="S470" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37067,7 +37067,7 @@
       </c>
       <c r="S471" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37146,7 +37146,7 @@
       </c>
       <c r="S472" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37225,7 +37225,7 @@
       </c>
       <c r="S473" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37300,7 +37300,7 @@
       </c>
       <c r="S474" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37379,7 +37379,7 @@
       </c>
       <c r="S475" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37458,7 +37458,7 @@
       </c>
       <c r="S476" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:48+00:00</t>
+          <t>2026-07-09T11:28:34+00:00</t>
         </is>
       </c>
     </row>
@@ -37537,7 +37537,7 @@
       </c>
       <c r="S477" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -37616,7 +37616,7 @@
       </c>
       <c r="S478" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -37695,7 +37695,7 @@
       </c>
       <c r="S479" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -37774,7 +37774,7 @@
       </c>
       <c r="S480" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -37853,7 +37853,7 @@
       </c>
       <c r="S481" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -37932,7 +37932,7 @@
       </c>
       <c r="S482" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38011,7 +38011,7 @@
       </c>
       <c r="S483" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38090,7 +38090,7 @@
       </c>
       <c r="S484" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38169,7 +38169,7 @@
       </c>
       <c r="S485" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38248,7 +38248,7 @@
       </c>
       <c r="S486" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38327,7 +38327,7 @@
       </c>
       <c r="S487" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38406,7 +38406,7 @@
       </c>
       <c r="S488" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38485,7 +38485,7 @@
       </c>
       <c r="S489" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38564,7 +38564,7 @@
       </c>
       <c r="S490" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38643,7 +38643,7 @@
       </c>
       <c r="S491" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38722,7 +38722,7 @@
       </c>
       <c r="S492" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38801,7 +38801,7 @@
       </c>
       <c r="S493" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38880,7 +38880,7 @@
       </c>
       <c r="S494" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -38959,7 +38959,7 @@
       </c>
       <c r="S495" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       </c>
       <c r="S496" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:51+00:00</t>
+          <t>2026-07-09T11:28:38+00:00</t>
         </is>
       </c>
     </row>
@@ -39117,7 +39117,7 @@
       </c>
       <c r="S497" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39192,7 +39192,7 @@
       </c>
       <c r="S498" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39267,7 +39267,7 @@
       </c>
       <c r="S499" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39346,7 +39346,7 @@
       </c>
       <c r="S500" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39425,7 +39425,7 @@
       </c>
       <c r="S501" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39504,7 +39504,7 @@
       </c>
       <c r="S502" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39583,7 +39583,7 @@
       </c>
       <c r="S503" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39662,7 +39662,7 @@
       </c>
       <c r="S504" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39741,7 +39741,7 @@
       </c>
       <c r="S505" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39820,7 +39820,7 @@
       </c>
       <c r="S506" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39895,7 +39895,7 @@
       </c>
       <c r="S507" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -39974,7 +39974,7 @@
       </c>
       <c r="S508" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40049,7 +40049,7 @@
       </c>
       <c r="S509" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40128,7 +40128,7 @@
       </c>
       <c r="S510" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40207,7 +40207,7 @@
       </c>
       <c r="S511" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40282,7 +40282,7 @@
       </c>
       <c r="S512" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40361,7 +40361,7 @@
       </c>
       <c r="S513" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40440,7 +40440,7 @@
       </c>
       <c r="S514" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40519,7 +40519,7 @@
       </c>
       <c r="S515" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:53+00:00</t>
+          <t>2026-07-09T11:28:41+00:00</t>
         </is>
       </c>
     </row>
@@ -40598,7 +40598,7 @@
       </c>
       <c r="S516" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -40677,7 +40677,7 @@
       </c>
       <c r="S517" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -40756,7 +40756,7 @@
       </c>
       <c r="S518" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -40835,7 +40835,7 @@
       </c>
       <c r="S519" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -40914,7 +40914,7 @@
       </c>
       <c r="S520" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -40989,7 +40989,7 @@
       </c>
       <c r="S521" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41068,7 +41068,7 @@
       </c>
       <c r="S522" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41147,7 +41147,7 @@
       </c>
       <c r="S523" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41226,7 +41226,7 @@
       </c>
       <c r="S524" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41301,7 +41301,7 @@
       </c>
       <c r="S525" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41376,7 +41376,7 @@
       </c>
       <c r="S526" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41455,7 +41455,7 @@
       </c>
       <c r="S527" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41530,7 +41530,7 @@
       </c>
       <c r="S528" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41609,7 +41609,7 @@
       </c>
       <c r="S529" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41684,7 +41684,7 @@
       </c>
       <c r="S530" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41763,7 +41763,7 @@
       </c>
       <c r="S531" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41842,7 +41842,7 @@
       </c>
       <c r="S532" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -41921,7 +41921,7 @@
       </c>
       <c r="S533" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:56+00:00</t>
+          <t>2026-07-09T11:28:44+00:00</t>
         </is>
       </c>
     </row>
@@ -42000,7 +42000,7 @@
       </c>
       <c r="S534" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:59+00:00</t>
+          <t>2026-07-09T11:28:47+00:00</t>
         </is>
       </c>
     </row>
@@ -42075,7 +42075,7 @@
       </c>
       <c r="S535" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:59+00:00</t>
+          <t>2026-07-09T11:28:47+00:00</t>
         </is>
       </c>
     </row>
@@ -42154,7 +42154,7 @@
       </c>
       <c r="S536" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:59+00:00</t>
+          <t>2026-07-09T11:28:47+00:00</t>
         </is>
       </c>
     </row>
@@ -42233,7 +42233,7 @@
       </c>
       <c r="S537" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:59+00:00</t>
+          <t>2026-07-09T11:28:47+00:00</t>
         </is>
       </c>
     </row>
@@ -42312,7 +42312,7 @@
       </c>
       <c r="S538" t="inlineStr">
         <is>
-          <t>2026-07-09T10:13:59+00:00</t>
+          <t>2026-07-09T11:28:47+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>